<commit_message>
feat: Implement core VFlexP power system modeling components in separate .slx files, functions, and data, updating install script and gitignore.
</commit_message>
<xml_diff>
--- a/bus_systems/VSM_and_SG.xlsx
+++ b/bus_systems/VSM_and_SG.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://upcomillas-my.sharepoint.com/personal/atomas_comillas_edu/Documents/GitHub/VFlexP/bus_systems/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBB9C485-9A39-453A-913D-6A7114CC9CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{FBB9C485-9A39-453A-913D-6A7114CC9CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12BD5097-F328-4770-85FA-E4EDB741D7B0}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus data" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="73">
   <si>
     <t>bus_i</t>
   </si>
@@ -112,15 +112,6 @@
     <t>series RL static omega</t>
   </si>
   <si>
-    <t>Complexity_bus_LF</t>
-  </si>
-  <si>
-    <t>Complexity_load_LF</t>
-  </si>
-  <si>
-    <t>PQ</t>
-  </si>
-  <si>
     <t>fbus</t>
   </si>
   <si>
@@ -170,12 +161,6 @@
   </si>
   <si>
     <t>Complexity</t>
-  </si>
-  <si>
-    <t>Complexity_LF</t>
-  </si>
-  <si>
-    <t>static omega</t>
   </si>
   <si>
     <t>bus</t>
@@ -625,28 +610,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.42578125" customWidth="1"/>
-    <col min="2" max="2" width="4.5703125" customWidth="1"/>
-    <col min="3" max="3" width="4.140625" customWidth="1"/>
-    <col min="4" max="4" width="3.42578125" customWidth="1"/>
-    <col min="5" max="6" width="6.42578125" customWidth="1"/>
-    <col min="7" max="7" width="4.5703125" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" customWidth="1"/>
-    <col min="10" max="10" width="6.85546875" customWidth="1"/>
-    <col min="11" max="11" width="4.85546875" customWidth="1"/>
-    <col min="12" max="12" width="5.5703125" customWidth="1"/>
-    <col min="13" max="13" width="5.140625" customWidth="1"/>
-    <col min="14" max="14" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="5.44140625" customWidth="1"/>
+    <col min="2" max="2" width="4.5546875" customWidth="1"/>
+    <col min="3" max="3" width="4.109375" customWidth="1"/>
+    <col min="4" max="4" width="3.44140625" customWidth="1"/>
+    <col min="5" max="6" width="6.44140625" customWidth="1"/>
+    <col min="7" max="7" width="4.5546875" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" customWidth="1"/>
+    <col min="9" max="9" width="13.109375" customWidth="1"/>
+    <col min="10" max="10" width="6.88671875" customWidth="1"/>
+    <col min="11" max="11" width="4.88671875" customWidth="1"/>
+    <col min="12" max="12" width="5.5546875" customWidth="1"/>
+    <col min="13" max="13" width="5.109375" customWidth="1"/>
+    <col min="14" max="14" width="14.109375" customWidth="1"/>
     <col min="15" max="15" width="19" customWidth="1"/>
-    <col min="16" max="16" width="16.85546875" customWidth="1"/>
-    <col min="17" max="17" width="17.5703125" customWidth="1"/>
+    <col min="16" max="16" width="16.88671875" customWidth="1"/>
+    <col min="17" max="17" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -692,14 +677,8 @@
       <c r="O1" t="s">
         <v>27</v>
       </c>
-      <c r="P1" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>30</v>
-      </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -745,14 +724,8 @@
       <c r="O2" t="s">
         <v>28</v>
       </c>
-      <c r="P2" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>31</v>
-      </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -797,12 +770,6 @@
       </c>
       <c r="O3" t="s">
         <v>28</v>
-      </c>
-      <c r="P3" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -812,71 +779,68 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="4.5703125" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" customWidth="1"/>
-    <col min="4" max="4" width="4.42578125" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="8" width="5.42578125" customWidth="1"/>
-    <col min="9" max="9" width="4.85546875" customWidth="1"/>
-    <col min="10" max="10" width="5.42578125" customWidth="1"/>
-    <col min="11" max="11" width="5.85546875" customWidth="1"/>
-    <col min="12" max="12" width="7.140625" customWidth="1"/>
-    <col min="13" max="13" width="7.42578125" customWidth="1"/>
-    <col min="14" max="14" width="10.140625" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" customWidth="1"/>
+    <col min="1" max="2" width="4.5546875" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" customWidth="1"/>
+    <col min="4" max="4" width="4.44140625" customWidth="1"/>
+    <col min="5" max="5" width="5.33203125" customWidth="1"/>
+    <col min="6" max="8" width="5.44140625" customWidth="1"/>
+    <col min="9" max="9" width="4.88671875" customWidth="1"/>
+    <col min="10" max="10" width="5.44140625" customWidth="1"/>
+    <col min="11" max="11" width="5.88671875" customWidth="1"/>
+    <col min="12" max="12" width="7.109375" customWidth="1"/>
+    <col min="13" max="13" width="7.44140625" customWidth="1"/>
+    <col min="14" max="14" width="10.109375" customWidth="1"/>
+    <col min="15" max="15" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" t="s">
         <v>39</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>41</v>
       </c>
-      <c r="J1" t="s">
-        <v>42</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>43</v>
       </c>
-      <c r="L1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M1" t="s">
-        <v>46</v>
-      </c>
       <c r="N1" t="s">
-        <v>48</v>
-      </c>
-      <c r="O1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -893,13 +857,13 @@
         <v>0.03</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I2" t="s">
         <v>5</v>
@@ -911,16 +875,13 @@
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="M2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N2" t="s">
         <v>26</v>
-      </c>
-      <c r="O2" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -931,121 +892,121 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:V3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.85546875" customWidth="1"/>
-    <col min="2" max="2" width="4.5703125" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="5.85546875" customWidth="1"/>
-    <col min="6" max="6" width="5.42578125" customWidth="1"/>
-    <col min="7" max="8" width="6.42578125" customWidth="1"/>
-    <col min="9" max="9" width="5.85546875" customWidth="1"/>
-    <col min="10" max="10" width="5.42578125" customWidth="1"/>
-    <col min="11" max="11" width="5.140625" customWidth="1"/>
-    <col min="12" max="13" width="3.7109375" customWidth="1"/>
-    <col min="14" max="14" width="7.28515625" customWidth="1"/>
-    <col min="15" max="15" width="7.5703125" customWidth="1"/>
-    <col min="16" max="16" width="7.28515625" customWidth="1"/>
-    <col min="17" max="17" width="7.5703125" customWidth="1"/>
-    <col min="18" max="18" width="9.140625" customWidth="1"/>
-    <col min="19" max="20" width="8.42578125" customWidth="1"/>
-    <col min="21" max="21" width="7.42578125" customWidth="1"/>
-    <col min="22" max="22" width="3.5703125" customWidth="1"/>
+    <col min="1" max="1" width="3.88671875" customWidth="1"/>
+    <col min="2" max="2" width="4.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="5.88671875" customWidth="1"/>
+    <col min="6" max="6" width="5.44140625" customWidth="1"/>
+    <col min="7" max="8" width="6.44140625" customWidth="1"/>
+    <col min="9" max="9" width="5.88671875" customWidth="1"/>
+    <col min="10" max="10" width="5.44140625" customWidth="1"/>
+    <col min="11" max="11" width="5.109375" customWidth="1"/>
+    <col min="12" max="13" width="3.6640625" customWidth="1"/>
+    <col min="14" max="14" width="7.33203125" customWidth="1"/>
+    <col min="15" max="15" width="7.5546875" customWidth="1"/>
+    <col min="16" max="16" width="7.33203125" customWidth="1"/>
+    <col min="17" max="17" width="7.5546875" customWidth="1"/>
+    <col min="18" max="18" width="9.109375" customWidth="1"/>
+    <col min="19" max="20" width="8.44140625" customWidth="1"/>
+    <col min="21" max="21" width="7.44140625" customWidth="1"/>
+    <col min="22" max="22" width="3.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" t="s">
         <v>53</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" t="s">
         <v>55</v>
       </c>
-      <c r="F1" t="s">
+      <c r="K1" t="s">
         <v>56</v>
       </c>
-      <c r="G1" t="s">
+      <c r="L1" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" t="s">
         <v>58</v>
       </c>
-      <c r="H1" t="s">
+      <c r="N1" t="s">
         <v>59</v>
       </c>
-      <c r="I1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="O1" t="s">
         <v>60</v>
       </c>
-      <c r="K1" t="s">
+      <c r="P1" t="s">
         <v>61</v>
       </c>
-      <c r="L1" t="s">
+      <c r="Q1" t="s">
         <v>62</v>
       </c>
-      <c r="M1" t="s">
+      <c r="R1" t="s">
         <v>63</v>
       </c>
-      <c r="N1" t="s">
+      <c r="S1" t="s">
         <v>64</v>
       </c>
-      <c r="O1" t="s">
+      <c r="T1" t="s">
         <v>65</v>
       </c>
-      <c r="P1" t="s">
+      <c r="U1" t="s">
         <v>66</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="V1" t="s">
         <v>67</v>
       </c>
-      <c r="R1" t="s">
-        <v>68</v>
-      </c>
-      <c r="S1" t="s">
-        <v>69</v>
-      </c>
-      <c r="T1" t="s">
-        <v>70</v>
-      </c>
-      <c r="U1" t="s">
-        <v>71</v>
-      </c>
-      <c r="V1" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C2">
         <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E2" t="s">
         <v>2</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I2" t="s">
         <v>1</v>
@@ -1090,12 +1051,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C3">
         <v>80</v>
@@ -1113,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I3" t="s">
         <v>1</v>
@@ -1166,24 +1127,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.85546875" customWidth="1"/>
-    <col min="2" max="3" width="2.85546875" customWidth="1"/>
+    <col min="1" max="1" width="4.88671875" customWidth="1"/>
+    <col min="2" max="3" width="2.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1191,7 +1152,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>